<commit_message>
Update & execute test cases
</commit_message>
<xml_diff>
--- a/Test.xlsx
+++ b/Test.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet name="Test Strategy" sheetId="1" state="visible" r:id="rId3"/>
@@ -17,6 +17,14 @@
     <sheet name="Bug Report" sheetId="7" state="visible" r:id="rId9"/>
     <sheet name="Test Metrics" sheetId="8" state="visible" r:id="rId10"/>
   </sheets>
+  <definedNames>
+    <definedName function="false" hidden="true" localSheetId="6" name="_xlnm._FilterDatabase" vbProcedure="false">'Bug Report'!$B$5:$P$5</definedName>
+    <definedName function="false" hidden="true" localSheetId="4" name="_xlnm._FilterDatabase" vbProcedure="false">'Test Cases'!$B$5:$O$13</definedName>
+    <definedName function="false" hidden="true" localSheetId="7" name="_xlnm._FilterDatabase" vbProcedure="false">'Test Metrics'!$B$5:$D$21</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'Test Plan'!$B$5:$C$13</definedName>
+    <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">'Test Scenarios'!$B$5:$F$31</definedName>
+    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">'Test Strategy'!$B$6:$C$19</definedName>
+  </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
@@ -27,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="305" uniqueCount="219">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="324" uniqueCount="226">
   <si>
     <t xml:space="preserve">Test Strategy</t>
   </si>
@@ -44,40 +52,13 @@
     <t xml:space="preserve">Project Name</t>
   </si>
   <si>
-    <t xml:space="preserve">SQA Automation Portfolio Project: Swag Labs E-commerce Application</t>
+    <t xml:space="preserve">Swag Labs E-commerce Application</t>
   </si>
   <si>
     <t xml:space="preserve">Application Under Test (AUT)</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Swag Labs (</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">https://www.saucedemo.com/</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">)</t>
-    </r>
+    <t xml:space="preserve">Swag Labs (https://www.saucedemo.com/)</t>
   </si>
   <si>
     <t xml:space="preserve">Objective</t>
@@ -624,6 +605,9 @@
     <t xml:space="preserve">Priority</t>
   </si>
   <si>
+    <t xml:space="preserve">Test Cases Count</t>
+  </si>
+  <si>
     <t xml:space="preserve">TS_001</t>
   </si>
   <si>
@@ -866,7 +850,16 @@
     <t xml:space="preserve">User should be redirected to Inventory page. URL contains /inventory.html. "Products" title is visible.</t>
   </si>
   <si>
-    <t xml:space="preserve">You</t>
+    <t xml:space="preserve">User redirected to inventory page.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pass</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sharif Jobayed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">21/05/2025</t>
   </si>
   <si>
     <t xml:space="preserve">Functional</t>
@@ -889,6 +882,9 @@
     <t xml:space="preserve">Error message "Epic sadface: Username and password do not match any user in this service" should be displayed.</t>
   </si>
   <si>
+    <t xml:space="preserve">Error displayed</t>
+  </si>
+  <si>
     <t xml:space="preserve">TC_002_02</t>
   </si>
   <si>
@@ -930,6 +926,10 @@
     <t xml:space="preserve">"Remove" button should appear instead of "Add to cart". Shopping cart icon should show "1".</t>
   </si>
   <si>
+    <t xml:space="preserve">- Remove button appeared
+- Item count in cart displayed</t>
+  </si>
+  <si>
     <t xml:space="preserve">Black-Box</t>
   </si>
   <si>
@@ -948,6 +948,10 @@
   </si>
   <si>
     <t xml:space="preserve">Item should be removed from cart. Shopping cart icon should show "0".</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- Item removed
+- Count updated</t>
   </si>
   <si>
     <t xml:space="preserve">TC_019_01</t>
@@ -1000,25 +1004,7 @@
     <t xml:space="preserve">Bug Report</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="12"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Bug </t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="12"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve">ID</t>
-    </r>
+    <t xml:space="preserve">Bug ID</t>
   </si>
   <si>
     <t xml:space="preserve">Title</t>
@@ -1027,147 +1013,30 @@
     <t xml:space="preserve">Steps to Reproduce</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="12"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Severity
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="12"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve">(Critical / High / Medium / Low)</t>
-    </r>
+    <t xml:space="preserve">Severity
+(Critical / High / Medium / Low)</t>
   </si>
   <si>
     <t xml:space="preserve"> Priority (P1-P4) </t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="12"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Status
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="12"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve">(Open / In Progress / To Test / Closed / Reopened)</t>
-    </r>
+    <t xml:space="preserve">Status
+(Open / In Progress / To Test / Closed / Reopened)</t>
   </si>
   <si>
     <t xml:space="preserve">Media (Image / Screencast)</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="12"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve">	Reported </t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="12"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">By</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="12"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve">Date </t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="12"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Reported</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="12"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve">Assigned </t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="12"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">To </t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="12"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve">(Simulated Dev)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="12"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve"> Fix </t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="12"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve">Version (Simulated)</t>
-    </r>
+    <t xml:space="preserve">	Reported By</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Date Reported</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Assigned To (Simulated Dev)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Fix Version (Simulated)</t>
   </si>
   <si>
     <t xml:space="preserve"> Comments</t>
@@ -1291,7 +1160,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="0.00%"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="11">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -1353,17 +1222,12 @@
       <charset val="1"/>
     </font>
     <font>
+      <b val="true"/>
       <sz val="12"/>
       <color rgb="FF0000FF"/>
       <name val="Times New Roman"/>
       <family val="1"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <b val="true"/>
-      <sz val="12"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
     </font>
   </fonts>
   <fills count="3">
@@ -1414,7 +1278,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="21">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1459,59 +1323,43 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1524,6 +1372,23 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
+  <dxfs count="2">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFDDDDDD"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <colors>
     <indexedColors>
       <rgbColor rgb="FF000000"/>
@@ -1585,6 +1450,30 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+</file>
+
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+</file>
+
+<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+</file>
+
+<file path=xl/drawings/drawing6.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1744,7 +1633,7 @@
       <c r="B8" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="C8" s="11" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1760,7 +1649,7 @@
       <c r="B10" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C10" s="11" t="s">
+      <c r="C10" s="12" t="s">
         <v>11</v>
       </c>
     </row>
@@ -1776,7 +1665,7 @@
       <c r="B12" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="C12" s="11" t="s">
+      <c r="C12" s="12" t="s">
         <v>15</v>
       </c>
     </row>
@@ -1784,7 +1673,7 @@
       <c r="B13" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="C13" s="11" t="s">
+      <c r="C13" s="12" t="s">
         <v>17</v>
       </c>
     </row>
@@ -1792,7 +1681,7 @@
       <c r="B14" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="C14" s="11" t="s">
+      <c r="C14" s="12" t="s">
         <v>19</v>
       </c>
     </row>
@@ -1824,7 +1713,7 @@
       <c r="B18" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="C18" s="11" t="s">
+      <c r="C18" s="12" t="s">
         <v>27</v>
       </c>
     </row>
@@ -1832,17 +1721,18 @@
       <c r="B19" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="C19" s="11" t="s">
+      <c r="C19" s="12" t="s">
         <v>29</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="B6:C19"/>
   <mergeCells count="2">
     <mergeCell ref="B3:C3"/>
     <mergeCell ref="B4:C4"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="C8" r:id="rId1" display="https://www.saucedemo.com/"/>
+    <hyperlink ref="C8" r:id="rId1" display="Swag Labs (https://www.saucedemo.com/)"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
@@ -1851,6 +1741,7 @@
     <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
     <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
   </headerFooter>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -1862,91 +1753,92 @@
   <dimension ref="B3:C13"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1" min="1" style="12" width="11.53"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="11.53"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="13" width="17.24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="12" width="50.08"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="4" style="12" width="11.53"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="50.08"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="4" style="1" width="11.53"/>
   </cols>
   <sheetData>
     <row r="3" customFormat="false" ht="22.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B3" s="14" t="s">
+      <c r="B3" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="C3" s="14"/>
+      <c r="C3" s="5"/>
     </row>
     <row r="5" s="13" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B5" s="15" t="s">
+      <c r="B5" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="C5" s="15" t="s">
+      <c r="C5" s="10" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B6" s="16" t="s">
+      <c r="B6" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="C6" s="17" t="s">
+      <c r="C6" s="12" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B7" s="16" t="s">
+      <c r="B7" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="C7" s="18" t="s">
+      <c r="C7" s="3" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="64.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B8" s="16" t="s">
+      <c r="B8" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="C8" s="18" t="s">
+      <c r="C8" s="3" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B9" s="16" t="s">
+      <c r="B9" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="C9" s="18" t="s">
+      <c r="C9" s="3" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="77.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B10" s="16" t="s">
+    <row r="10" customFormat="false" ht="64.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B10" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="C10" s="17" t="s">
+      <c r="C10" s="12" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B11" s="16" t="s">
+      <c r="B11" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="C11" s="18" t="s">
+      <c r="C11" s="3" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B12" s="16" t="s">
+      <c r="B12" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="C12" s="18" t="s">
+      <c r="C12" s="3" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B13" s="16" t="s">
+      <c r="B13" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="C13" s="18" t="s">
+      <c r="C13" s="3" t="s">
         <v>46</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="B5:C13"/>
   <mergeCells count="1">
     <mergeCell ref="B3:C3"/>
   </mergeCells>
@@ -1957,6 +1849,7 @@
     <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
     <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
   </headerFooter>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -1965,404 +1858,430 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="B3:E31"/>
+  <dimension ref="B3:F31"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1" min="1" style="12" width="11.53"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="11.53"/>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="2" min="2" style="13" width="11.53"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="12" width="22.53"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="12" width="36.87"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="22.53"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="36.88"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="13" width="14.88"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="6" style="12" width="11.53"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="13" width="14.6"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="7" style="1" width="11.53"/>
   </cols>
   <sheetData>
     <row r="3" customFormat="false" ht="22.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B3" s="14" t="s">
+      <c r="B3" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="C3" s="14"/>
-      <c r="D3" s="14"/>
-      <c r="E3" s="14"/>
+      <c r="C3" s="5"/>
+      <c r="D3" s="5"/>
+      <c r="E3" s="5"/>
     </row>
     <row r="5" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B5" s="15" t="s">
+      <c r="B5" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="C5" s="15" t="s">
+      <c r="C5" s="10" t="s">
         <v>49</v>
       </c>
-      <c r="D5" s="15" t="s">
+      <c r="D5" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="E5" s="15" t="s">
+      <c r="E5" s="10" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F5" s="10" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="13" t="s">
-        <v>52</v>
-      </c>
-      <c r="C6" s="12" t="s">
         <v>53</v>
       </c>
-      <c r="D6" s="12" t="s">
+      <c r="C6" s="1" t="s">
         <v>54</v>
       </c>
+      <c r="D6" s="1" t="s">
+        <v>55</v>
+      </c>
       <c r="E6" s="13" t="s">
-        <v>55</v>
+        <v>56</v>
+      </c>
+      <c r="F6" s="13" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="E7" s="13" t="s">
         <v>56</v>
       </c>
-      <c r="C7" s="12" t="s">
-        <v>53</v>
-      </c>
-      <c r="D7" s="12" t="s">
-        <v>57</v>
-      </c>
-      <c r="E7" s="13" t="s">
-        <v>55</v>
+      <c r="F7" s="13" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="13" t="s">
-        <v>58</v>
-      </c>
-      <c r="C8" s="12" t="s">
-        <v>53</v>
-      </c>
-      <c r="D8" s="12" t="s">
         <v>59</v>
       </c>
+      <c r="C8" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>60</v>
+      </c>
       <c r="E8" s="13" t="s">
-        <v>55</v>
+        <v>56</v>
+      </c>
+      <c r="F8" s="13" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="13" t="s">
-        <v>60</v>
-      </c>
-      <c r="C9" s="12" t="s">
-        <v>53</v>
-      </c>
-      <c r="D9" s="12" t="s">
         <v>61</v>
       </c>
+      <c r="C9" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>62</v>
+      </c>
       <c r="E9" s="13" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="13" t="s">
-        <v>62</v>
-      </c>
-      <c r="C10" s="12" t="s">
         <v>63</v>
       </c>
-      <c r="D10" s="12" t="s">
+      <c r="C10" s="1" t="s">
         <v>64</v>
       </c>
+      <c r="D10" s="1" t="s">
+        <v>65</v>
+      </c>
       <c r="E10" s="13" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="13" t="s">
+        <v>67</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="E11" s="13" t="s">
         <v>66</v>
-      </c>
-      <c r="C11" s="12" t="s">
-        <v>63</v>
-      </c>
-      <c r="D11" s="12" t="s">
-        <v>67</v>
-      </c>
-      <c r="E11" s="13" t="s">
-        <v>65</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="13" t="s">
-        <v>68</v>
-      </c>
-      <c r="C12" s="12" t="s">
-        <v>63</v>
-      </c>
-      <c r="D12" s="12" t="s">
         <v>69</v>
       </c>
+      <c r="C12" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>70</v>
+      </c>
       <c r="E12" s="13" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="13" t="s">
-        <v>70</v>
-      </c>
-      <c r="C13" s="12" t="s">
-        <v>63</v>
-      </c>
-      <c r="D13" s="12" t="s">
         <v>71</v>
       </c>
+      <c r="C13" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>72</v>
+      </c>
       <c r="E13" s="13" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="13" t="s">
-        <v>72</v>
-      </c>
-      <c r="C14" s="12" t="s">
-        <v>63</v>
-      </c>
-      <c r="D14" s="12" t="s">
         <v>73</v>
       </c>
+      <c r="C14" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>74</v>
+      </c>
       <c r="E14" s="13" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="13" t="s">
-        <v>74</v>
-      </c>
-      <c r="C15" s="12" t="s">
         <v>75</v>
       </c>
-      <c r="D15" s="12" t="s">
+      <c r="C15" s="1" t="s">
         <v>76</v>
       </c>
+      <c r="D15" s="1" t="s">
+        <v>77</v>
+      </c>
       <c r="E15" s="13" t="s">
-        <v>55</v>
+        <v>56</v>
+      </c>
+      <c r="F15" s="13" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="13" t="s">
-        <v>77</v>
-      </c>
-      <c r="C16" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="D16" s="12" t="s">
         <v>78</v>
       </c>
+      <c r="C16" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>79</v>
+      </c>
       <c r="E16" s="13" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="13" t="s">
-        <v>79</v>
-      </c>
-      <c r="C17" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="D17" s="12" t="s">
         <v>80</v>
       </c>
+      <c r="C17" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>81</v>
+      </c>
       <c r="E17" s="13" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="13" t="s">
-        <v>81</v>
-      </c>
-      <c r="C18" s="12" t="s">
         <v>82</v>
       </c>
-      <c r="D18" s="12" t="s">
+      <c r="C18" s="1" t="s">
         <v>83</v>
       </c>
+      <c r="D18" s="1" t="s">
+        <v>84</v>
+      </c>
       <c r="E18" s="13" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="13" t="s">
-        <v>84</v>
-      </c>
-      <c r="C19" s="12" t="s">
-        <v>82</v>
-      </c>
-      <c r="D19" s="12" t="s">
         <v>85</v>
       </c>
+      <c r="C19" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>86</v>
+      </c>
       <c r="E19" s="13" t="s">
-        <v>55</v>
+        <v>56</v>
+      </c>
+      <c r="F19" s="13" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="13" t="s">
-        <v>86</v>
-      </c>
-      <c r="C20" s="12" t="s">
-        <v>82</v>
-      </c>
-      <c r="D20" s="12" t="s">
         <v>87</v>
       </c>
+      <c r="C20" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>88</v>
+      </c>
       <c r="E20" s="13" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="13" t="s">
-        <v>88</v>
-      </c>
-      <c r="C21" s="12" t="s">
         <v>89</v>
       </c>
-      <c r="D21" s="12" t="s">
+      <c r="C21" s="1" t="s">
         <v>90</v>
       </c>
+      <c r="D21" s="1" t="s">
+        <v>91</v>
+      </c>
       <c r="E21" s="13" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="13" t="s">
-        <v>91</v>
-      </c>
-      <c r="C22" s="12" t="s">
-        <v>89</v>
-      </c>
-      <c r="D22" s="12" t="s">
         <v>92</v>
       </c>
+      <c r="C22" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>93</v>
+      </c>
       <c r="E22" s="13" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="13" t="s">
-        <v>93</v>
-      </c>
-      <c r="C23" s="12" t="s">
-        <v>89</v>
-      </c>
-      <c r="D23" s="12" t="s">
         <v>94</v>
       </c>
+      <c r="C23" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="D23" s="1" t="s">
+        <v>95</v>
+      </c>
       <c r="E23" s="13" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="13" t="s">
-        <v>95</v>
-      </c>
-      <c r="C24" s="12" t="s">
-        <v>89</v>
-      </c>
-      <c r="D24" s="12" t="s">
         <v>96</v>
       </c>
+      <c r="C24" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="D24" s="1" t="s">
+        <v>97</v>
+      </c>
       <c r="E24" s="13" t="s">
-        <v>55</v>
+        <v>56</v>
+      </c>
+      <c r="F24" s="13" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="13" t="s">
-        <v>97</v>
-      </c>
-      <c r="C25" s="12" t="s">
-        <v>89</v>
-      </c>
-      <c r="D25" s="12" t="s">
         <v>98</v>
       </c>
+      <c r="C25" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>99</v>
+      </c>
       <c r="E25" s="13" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="13" t="s">
-        <v>99</v>
-      </c>
-      <c r="C26" s="12" t="s">
-        <v>89</v>
-      </c>
-      <c r="D26" s="12" t="s">
         <v>100</v>
       </c>
+      <c r="C26" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="D26" s="1" t="s">
+        <v>101</v>
+      </c>
       <c r="E26" s="13" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="13" t="s">
-        <v>101</v>
-      </c>
-      <c r="C27" s="12" t="s">
         <v>102</v>
       </c>
-      <c r="D27" s="12" t="s">
+      <c r="C27" s="1" t="s">
         <v>103</v>
       </c>
+      <c r="D27" s="1" t="s">
+        <v>104</v>
+      </c>
       <c r="E27" s="13" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="13" t="s">
+        <v>106</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="D28" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="E28" s="13" t="s">
         <v>105</v>
       </c>
-      <c r="C28" s="12" t="s">
-        <v>102</v>
-      </c>
-      <c r="D28" s="12" t="s">
-        <v>106</v>
-      </c>
-      <c r="E28" s="13" t="s">
-        <v>104</v>
+      <c r="F28" s="13" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B29" s="13" t="s">
-        <v>107</v>
-      </c>
-      <c r="C29" s="12" t="s">
-        <v>102</v>
-      </c>
-      <c r="D29" s="12" t="s">
         <v>108</v>
       </c>
+      <c r="C29" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="D29" s="1" t="s">
+        <v>109</v>
+      </c>
       <c r="E29" s="13" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B30" s="13" t="s">
-        <v>109</v>
-      </c>
-      <c r="C30" s="12" t="s">
         <v>110</v>
       </c>
-      <c r="D30" s="12" t="s">
+      <c r="C30" s="1" t="s">
         <v>111</v>
       </c>
+      <c r="D30" s="1" t="s">
+        <v>112</v>
+      </c>
       <c r="E30" s="13" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B31" s="13" t="s">
-        <v>112</v>
-      </c>
-      <c r="C31" s="12" t="s">
-        <v>110</v>
-      </c>
-      <c r="D31" s="12" t="s">
         <v>113</v>
       </c>
+      <c r="C31" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="D31" s="1" t="s">
+        <v>114</v>
+      </c>
       <c r="E31" s="13" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="B5:F31"/>
   <mergeCells count="1">
     <mergeCell ref="B3:E3"/>
   </mergeCells>
@@ -2373,6 +2292,7 @@
     <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
     <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
   </headerFooter>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -2402,334 +2322,396 @@
   <dimension ref="B3:O13"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1" min="1" style="12" width="11.53"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="6.12"/>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="3" min="2" style="13" width="11.53"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="12" width="18.78"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="12" width="22.81"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="12" width="32.55"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="12" width="26.43"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="8" style="12" width="11.53"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="18.79"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="22.81"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="32.55"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="26.43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="25.46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="13" width="14.05"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="27.41"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="12" min="11" style="13" width="11.53"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="13" width="14.19"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="13.91"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="1" width="15.44"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="16" style="1" width="11.53"/>
   </cols>
   <sheetData>
     <row r="3" customFormat="false" ht="22.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B3" s="14" t="s">
-        <v>114</v>
-      </c>
-      <c r="C3" s="14"/>
-      <c r="D3" s="14"/>
-      <c r="E3" s="14"/>
-      <c r="F3" s="14"/>
-      <c r="G3" s="14"/>
-      <c r="H3" s="14"/>
-      <c r="I3" s="14"/>
-      <c r="J3" s="14"/>
-      <c r="K3" s="14"/>
-      <c r="L3" s="14"/>
-      <c r="M3" s="14"/>
-      <c r="N3" s="14"/>
-      <c r="O3" s="14"/>
-    </row>
-    <row r="5" s="19" customFormat="true" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B5" s="15" t="s">
+      <c r="B3" s="5" t="s">
         <v>115</v>
       </c>
-      <c r="C5" s="15" t="s">
+      <c r="C3" s="5"/>
+      <c r="D3" s="5"/>
+      <c r="E3" s="5"/>
+      <c r="F3" s="5"/>
+      <c r="G3" s="5"/>
+      <c r="H3" s="5"/>
+      <c r="I3" s="5"/>
+      <c r="J3" s="5"/>
+      <c r="K3" s="5"/>
+      <c r="L3" s="5"/>
+      <c r="M3" s="5"/>
+      <c r="N3" s="5"/>
+      <c r="O3" s="5"/>
+    </row>
+    <row r="5" s="14" customFormat="true" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B5" s="10" t="s">
+        <v>116</v>
+      </c>
+      <c r="C5" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="D5" s="15" t="s">
-        <v>116</v>
-      </c>
-      <c r="E5" s="15" t="s">
+      <c r="D5" s="10" t="s">
         <v>117</v>
       </c>
-      <c r="F5" s="15" t="s">
+      <c r="E5" s="10" t="s">
         <v>118</v>
       </c>
-      <c r="G5" s="15" t="s">
+      <c r="F5" s="10" t="s">
         <v>119</v>
       </c>
-      <c r="H5" s="15" t="s">
+      <c r="G5" s="10" t="s">
         <v>120</v>
       </c>
-      <c r="I5" s="15" t="s">
+      <c r="H5" s="10" t="s">
         <v>121</v>
       </c>
-      <c r="J5" s="15" t="s">
+      <c r="I5" s="10" t="s">
         <v>122</v>
       </c>
-      <c r="K5" s="15" t="s">
+      <c r="J5" s="10" t="s">
+        <v>123</v>
+      </c>
+      <c r="K5" s="10" t="s">
         <v>51</v>
       </c>
-      <c r="L5" s="15" t="s">
-        <v>123</v>
-      </c>
-      <c r="M5" s="15" t="s">
+      <c r="L5" s="10" t="s">
         <v>124</v>
       </c>
-      <c r="N5" s="15" t="s">
+      <c r="M5" s="10" t="s">
         <v>125</v>
       </c>
-      <c r="O5" s="15" t="s">
+      <c r="N5" s="10" t="s">
         <v>126</v>
+      </c>
+      <c r="O5" s="10" t="s">
+        <v>127</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="64.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="13" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C6" s="13" t="s">
-        <v>52</v>
-      </c>
-      <c r="D6" s="12" t="s">
-        <v>128</v>
-      </c>
-      <c r="E6" s="12" t="s">
+        <v>53</v>
+      </c>
+      <c r="D6" s="1" t="s">
         <v>129</v>
       </c>
-      <c r="F6" s="12" t="s">
+      <c r="E6" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="G6" s="12" t="s">
+      <c r="F6" s="1" t="s">
         <v>131</v>
       </c>
-      <c r="K6" s="12" t="s">
-        <v>55</v>
-      </c>
-      <c r="L6" s="12" t="s">
+      <c r="G6" s="1" t="s">
         <v>132</v>
       </c>
-      <c r="N6" s="12" t="s">
+      <c r="H6" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="O6" s="12" t="s">
+      <c r="I6" s="13" t="s">
         <v>134</v>
+      </c>
+      <c r="K6" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="L6" s="13" t="s">
+        <v>135</v>
+      </c>
+      <c r="M6" s="13" t="s">
+        <v>136</v>
+      </c>
+      <c r="N6" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="O6" s="1" t="s">
+        <v>138</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="64.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="13" t="s">
+        <v>139</v>
+      </c>
+      <c r="C7" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="H7" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="I7" s="13" t="s">
+        <v>134</v>
+      </c>
+      <c r="K7" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="L7" s="13" t="s">
         <v>135</v>
       </c>
-      <c r="C7" s="13" t="s">
-        <v>56</v>
-      </c>
-      <c r="D7" s="12" t="s">
+      <c r="M7" s="13" t="s">
         <v>136</v>
       </c>
-      <c r="E7" s="12" t="s">
-        <v>129</v>
-      </c>
-      <c r="F7" s="12" t="s">
+      <c r="N7" s="1" t="s">
         <v>137</v>
       </c>
-      <c r="G7" s="12" t="s">
+      <c r="O7" s="1" t="s">
         <v>138</v>
-      </c>
-      <c r="K7" s="12" t="s">
-        <v>55</v>
-      </c>
-      <c r="L7" s="12" t="s">
-        <v>132</v>
-      </c>
-      <c r="N7" s="12" t="s">
-        <v>133</v>
-      </c>
-      <c r="O7" s="12" t="s">
-        <v>134</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="64.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="13" t="s">
-        <v>139</v>
+        <v>144</v>
       </c>
       <c r="C8" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="H8" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="I8" s="13" t="s">
+        <v>134</v>
+      </c>
+      <c r="K8" s="13" t="s">
         <v>56</v>
       </c>
-      <c r="D8" s="12" t="s">
-        <v>140</v>
-      </c>
-      <c r="E8" s="12" t="s">
-        <v>129</v>
-      </c>
-      <c r="F8" s="12" t="s">
-        <v>141</v>
-      </c>
-      <c r="G8" s="12" t="s">
+      <c r="L8" s="13" t="s">
+        <v>135</v>
+      </c>
+      <c r="M8" s="13" t="s">
+        <v>136</v>
+      </c>
+      <c r="N8" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="O8" s="1" t="s">
         <v>138</v>
-      </c>
-      <c r="K8" s="12" t="s">
-        <v>55</v>
-      </c>
-      <c r="L8" s="12" t="s">
-        <v>132</v>
-      </c>
-      <c r="N8" s="12" t="s">
-        <v>133</v>
-      </c>
-      <c r="O8" s="12" t="s">
-        <v>134</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="64.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="13" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="C9" s="13" t="s">
-        <v>58</v>
-      </c>
-      <c r="D9" s="12" t="s">
+        <v>59</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="H9" s="1" t="s">
         <v>143</v>
       </c>
-      <c r="E9" s="12" t="s">
-        <v>129</v>
-      </c>
-      <c r="F9" s="12" t="s">
-        <v>144</v>
-      </c>
-      <c r="G9" s="12" t="s">
-        <v>145</v>
-      </c>
-      <c r="K9" s="12" t="s">
-        <v>55</v>
-      </c>
-      <c r="L9" s="12" t="s">
-        <v>132</v>
-      </c>
-      <c r="N9" s="12" t="s">
-        <v>133</v>
-      </c>
-      <c r="O9" s="12" t="s">
+      <c r="I9" s="13" t="s">
         <v>134</v>
+      </c>
+      <c r="K9" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="L9" s="13" t="s">
+        <v>135</v>
+      </c>
+      <c r="M9" s="13" t="s">
+        <v>136</v>
+      </c>
+      <c r="N9" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="O9" s="1" t="s">
+        <v>138</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="13" t="s">
-        <v>146</v>
+        <v>151</v>
       </c>
       <c r="C10" s="13" t="s">
-        <v>74</v>
-      </c>
-      <c r="D10" s="12" t="s">
-        <v>147</v>
-      </c>
-      <c r="E10" s="12" t="s">
-        <v>148</v>
-      </c>
-      <c r="F10" s="12" t="s">
-        <v>149</v>
-      </c>
-      <c r="G10" s="12" t="s">
-        <v>150</v>
-      </c>
-      <c r="K10" s="12" t="s">
-        <v>55</v>
-      </c>
-      <c r="L10" s="12" t="s">
-        <v>132</v>
-      </c>
-      <c r="N10" s="12" t="s">
-        <v>133</v>
-      </c>
-      <c r="O10" s="12" t="s">
-        <v>151</v>
+        <v>75</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="G10" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="H10" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="I10" s="13" t="s">
+        <v>134</v>
+      </c>
+      <c r="K10" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="L10" s="13" t="s">
+        <v>135</v>
+      </c>
+      <c r="M10" s="13" t="s">
+        <v>136</v>
+      </c>
+      <c r="N10" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="O10" s="1" t="s">
+        <v>157</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="64.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="13" t="s">
-        <v>152</v>
+        <v>158</v>
       </c>
       <c r="C11" s="13" t="s">
-        <v>84</v>
-      </c>
-      <c r="D11" s="12" t="s">
-        <v>153</v>
-      </c>
-      <c r="E11" s="12" t="s">
-        <v>154</v>
-      </c>
-      <c r="F11" s="12" t="s">
-        <v>155</v>
-      </c>
-      <c r="G11" s="12" t="s">
-        <v>156</v>
-      </c>
-      <c r="K11" s="12" t="s">
-        <v>55</v>
-      </c>
-      <c r="L11" s="12" t="s">
-        <v>132</v>
-      </c>
-      <c r="N11" s="12" t="s">
-        <v>133</v>
-      </c>
-      <c r="O11" s="12" t="s">
-        <v>151</v>
+        <v>85</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="G11" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="H11" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="I11" s="13" t="s">
+        <v>134</v>
+      </c>
+      <c r="K11" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="L11" s="13" t="s">
+        <v>135</v>
+      </c>
+      <c r="M11" s="13" t="s">
+        <v>136</v>
+      </c>
+      <c r="N11" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="O11" s="1" t="s">
+        <v>157</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="115.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="13" t="s">
-        <v>157</v>
+        <v>164</v>
       </c>
       <c r="C12" s="13" t="s">
-        <v>95</v>
-      </c>
-      <c r="D12" s="12" t="s">
-        <v>158</v>
-      </c>
-      <c r="E12" s="12" t="s">
-        <v>159</v>
-      </c>
-      <c r="F12" s="12" t="s">
-        <v>160</v>
-      </c>
-      <c r="G12" s="12" t="s">
-        <v>161</v>
-      </c>
-      <c r="K12" s="12" t="s">
-        <v>55</v>
-      </c>
-      <c r="L12" s="12" t="s">
-        <v>132</v>
-      </c>
-      <c r="N12" s="12" t="s">
-        <v>133</v>
-      </c>
-      <c r="O12" s="12" t="s">
-        <v>162</v>
+        <v>96</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="G12" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="K12" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="L12" s="13" t="s">
+        <v>135</v>
+      </c>
+      <c r="N12" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="O12" s="1" t="s">
+        <v>169</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="64.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="13" t="s">
-        <v>163</v>
+        <v>170</v>
       </c>
       <c r="C13" s="13" t="s">
+        <v>106</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>171</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="F13" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="G13" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="K13" s="13" t="s">
         <v>105</v>
       </c>
-      <c r="D13" s="12" t="s">
-        <v>164</v>
-      </c>
-      <c r="E13" s="12" t="s">
-        <v>165</v>
-      </c>
-      <c r="F13" s="12" t="s">
-        <v>166</v>
-      </c>
-      <c r="G13" s="12" t="s">
-        <v>167</v>
-      </c>
-      <c r="K13" s="12" t="s">
-        <v>104</v>
-      </c>
-      <c r="L13" s="12" t="s">
-        <v>132</v>
-      </c>
-      <c r="N13" s="12" t="s">
-        <v>168</v>
-      </c>
-      <c r="O13" s="12" t="s">
-        <v>169</v>
+      <c r="L13" s="13" t="s">
+        <v>135</v>
+      </c>
+      <c r="N13" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="O13" s="1" t="s">
+        <v>176</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="B5:O13"/>
   <mergeCells count="1">
     <mergeCell ref="B3:O3"/>
   </mergeCells>
@@ -2740,6 +2722,7 @@
     <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
     <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
   </headerFooter>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -2769,92 +2752,95 @@
   <dimension ref="B3:BO5"/>
   <sheetFormatPr defaultColWidth="25.0390625" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="12" width="16.27"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="16.27"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="13" width="11.53"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="3" min="3" style="12" width="25.04"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="12" width="33.94"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="12" width="31.99"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="6" style="12" width="37.98"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="61" min="8" style="12" width="25.04"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="66" min="62" style="20" width="25.04"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="68" style="12" width="25.04"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="25.04"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="33.94"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="31.99"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="6" style="1" width="37.98"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="9" min="8" style="1" width="25.04"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="28.38"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="61" min="11" style="1" width="25.04"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="66" min="62" style="15" width="25.04"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="68" style="1" width="25.04"/>
   </cols>
   <sheetData>
     <row r="3" customFormat="false" ht="22.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B3" s="14" t="s">
-        <v>170</v>
-      </c>
-      <c r="C3" s="14"/>
-      <c r="D3" s="14"/>
-      <c r="E3" s="14"/>
-      <c r="F3" s="14"/>
-      <c r="G3" s="14"/>
-      <c r="H3" s="14"/>
-      <c r="I3" s="14"/>
-      <c r="J3" s="14"/>
-      <c r="K3" s="14"/>
-      <c r="L3" s="14"/>
-      <c r="M3" s="14"/>
-      <c r="N3" s="14"/>
-      <c r="O3" s="14"/>
-      <c r="P3" s="14"/>
-      <c r="Q3" s="14"/>
+      <c r="B3" s="5" t="s">
+        <v>177</v>
+      </c>
+      <c r="C3" s="5"/>
+      <c r="D3" s="5"/>
+      <c r="E3" s="5"/>
+      <c r="F3" s="5"/>
+      <c r="G3" s="5"/>
+      <c r="H3" s="5"/>
+      <c r="I3" s="5"/>
+      <c r="J3" s="5"/>
+      <c r="K3" s="5"/>
+      <c r="L3" s="5"/>
+      <c r="M3" s="5"/>
+      <c r="N3" s="5"/>
+      <c r="O3" s="5"/>
+      <c r="P3" s="5"/>
+      <c r="Q3" s="5"/>
     </row>
     <row r="5" s="13" customFormat="true" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B5" s="15" t="s">
-        <v>171</v>
-      </c>
-      <c r="C5" s="15" t="s">
-        <v>172</v>
-      </c>
-      <c r="D5" s="21" t="s">
+      <c r="B5" s="10" t="s">
+        <v>178</v>
+      </c>
+      <c r="C5" s="10" t="s">
+        <v>179</v>
+      </c>
+      <c r="D5" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="E5" s="21" t="s">
-        <v>173</v>
-      </c>
-      <c r="F5" s="15" t="s">
-        <v>119</v>
-      </c>
-      <c r="G5" s="15" t="s">
+      <c r="E5" s="10" t="s">
+        <v>180</v>
+      </c>
+      <c r="F5" s="10" t="s">
         <v>120</v>
       </c>
-      <c r="H5" s="15" t="s">
-        <v>174</v>
-      </c>
-      <c r="I5" s="21" t="s">
-        <v>175</v>
-      </c>
-      <c r="J5" s="15" t="s">
-        <v>176</v>
-      </c>
-      <c r="K5" s="15" t="s">
-        <v>177</v>
-      </c>
-      <c r="L5" s="21" t="s">
-        <v>178</v>
-      </c>
-      <c r="M5" s="21" t="s">
-        <v>179</v>
-      </c>
-      <c r="N5" s="21" t="s">
-        <v>180</v>
-      </c>
-      <c r="O5" s="15" t="s">
+      <c r="G5" s="10" t="s">
+        <v>121</v>
+      </c>
+      <c r="H5" s="10" t="s">
         <v>181</v>
       </c>
-      <c r="P5" s="15" t="s">
+      <c r="I5" s="10" t="s">
         <v>182</v>
       </c>
-      <c r="Q5" s="22"/>
-      <c r="BJ5" s="22"/>
-      <c r="BK5" s="22"/>
-      <c r="BL5" s="22"/>
-      <c r="BM5" s="22"/>
-      <c r="BN5" s="22"/>
-      <c r="BO5" s="0"/>
+      <c r="J5" s="10" t="s">
+        <v>183</v>
+      </c>
+      <c r="K5" s="10" t="s">
+        <v>184</v>
+      </c>
+      <c r="L5" s="10" t="s">
+        <v>185</v>
+      </c>
+      <c r="M5" s="10" t="s">
+        <v>186</v>
+      </c>
+      <c r="N5" s="10" t="s">
+        <v>187</v>
+      </c>
+      <c r="O5" s="10" t="s">
+        <v>188</v>
+      </c>
+      <c r="P5" s="10" t="s">
+        <v>189</v>
+      </c>
+      <c r="Q5" s="16"/>
+      <c r="BJ5" s="16"/>
+      <c r="BK5" s="16"/>
+      <c r="BL5" s="16"/>
+      <c r="BM5" s="16"/>
+      <c r="BN5" s="16"/>
+      <c r="BO5" s="17"/>
     </row>
   </sheetData>
+  <autoFilter ref="B5:P5"/>
   <mergeCells count="1">
     <mergeCell ref="B3:Q3"/>
   </mergeCells>
@@ -2865,6 +2851,7 @@
     <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
     <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
   </headerFooter>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -2873,201 +2860,203 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="B3:D21"/>
+  <dimension ref="A3:D21"/>
   <sheetFormatPr defaultColWidth="21.70703125" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="2" min="1" style="12" width="21.7"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="12" width="26.57"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="12" width="38.25"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="5" style="12" width="21.7"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="2" min="1" style="1" width="21.7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="26.57"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="38.25"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="5" style="1" width="21.7"/>
   </cols>
   <sheetData>
     <row r="3" customFormat="false" ht="22.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B3" s="14" t="s">
-        <v>183</v>
-      </c>
-      <c r="C3" s="14"/>
-      <c r="D3" s="14"/>
-    </row>
-    <row r="5" s="23" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B5" s="15" t="s">
-        <v>184</v>
-      </c>
-      <c r="C5" s="15" t="s">
-        <v>185</v>
-      </c>
-      <c r="D5" s="15" t="s">
-        <v>186</v>
+      <c r="B3" s="5" t="s">
+        <v>190</v>
+      </c>
+      <c r="C3" s="5"/>
+      <c r="D3" s="5"/>
+    </row>
+    <row r="5" s="19" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="18"/>
+      <c r="B5" s="10" t="s">
+        <v>191</v>
+      </c>
+      <c r="C5" s="10" t="s">
+        <v>192</v>
+      </c>
+      <c r="D5" s="10" t="s">
+        <v>193</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B6" s="17" t="s">
-        <v>187</v>
-      </c>
-      <c r="C6" s="18" t="s">
-        <v>188</v>
-      </c>
-      <c r="D6" s="18" t="s">
-        <v>189</v>
+      <c r="B6" s="12" t="s">
+        <v>194</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>195</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>196</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B7" s="17" t="s">
-        <v>190</v>
-      </c>
-      <c r="C7" s="18" t="n">
+      <c r="B7" s="12" t="s">
+        <v>197</v>
+      </c>
+      <c r="C7" s="3" t="n">
         <v>20</v>
       </c>
-      <c r="D7" s="18" t="s">
-        <v>191</v>
+      <c r="D7" s="3" t="s">
+        <v>198</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B8" s="17" t="s">
-        <v>192</v>
-      </c>
-      <c r="C8" s="18" t="n">
+      <c r="B8" s="12" t="s">
+        <v>199</v>
+      </c>
+      <c r="C8" s="3" t="n">
         <v>17</v>
       </c>
-      <c r="D8" s="18" t="s">
-        <v>193</v>
+      <c r="D8" s="3" t="s">
+        <v>200</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B9" s="17" t="s">
-        <v>194</v>
-      </c>
-      <c r="C9" s="18" t="n">
+      <c r="B9" s="12" t="s">
+        <v>201</v>
+      </c>
+      <c r="C9" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="D9" s="18" t="s">
-        <v>195</v>
+      <c r="D9" s="3" t="s">
+        <v>202</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B10" s="17" t="s">
-        <v>196</v>
-      </c>
-      <c r="C10" s="24" t="n">
+      <c r="B10" s="12" t="s">
+        <v>203</v>
+      </c>
+      <c r="C10" s="20" t="n">
         <v>0.85</v>
       </c>
-      <c r="D10" s="18" t="s">
-        <v>197</v>
+      <c r="D10" s="3" t="s">
+        <v>204</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B11" s="17" t="s">
-        <v>198</v>
-      </c>
-      <c r="C11" s="18" t="n">
+      <c r="B11" s="12" t="s">
+        <v>205</v>
+      </c>
+      <c r="C11" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="D11" s="18" t="s">
-        <v>199</v>
+      <c r="D11" s="3" t="s">
+        <v>206</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B12" s="17" t="s">
-        <v>200</v>
-      </c>
-      <c r="C12" s="18" t="n">
+      <c r="B12" s="12" t="s">
+        <v>207</v>
+      </c>
+      <c r="C12" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="D12" s="18" t="s">
-        <v>201</v>
+      <c r="D12" s="3" t="s">
+        <v>208</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B13" s="17" t="s">
-        <v>202</v>
-      </c>
-      <c r="C13" s="18" t="n">
+      <c r="B13" s="12" t="s">
+        <v>209</v>
+      </c>
+      <c r="C13" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="D13" s="18"/>
+      <c r="D13" s="3"/>
     </row>
     <row r="14" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B14" s="17" t="s">
-        <v>203</v>
-      </c>
-      <c r="C14" s="18" t="n">
+      <c r="B14" s="12" t="s">
+        <v>210</v>
+      </c>
+      <c r="C14" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="D14" s="18" t="s">
-        <v>204</v>
+      <c r="D14" s="3" t="s">
+        <v>211</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B15" s="17" t="s">
-        <v>205</v>
-      </c>
-      <c r="C15" s="18" t="n">
+      <c r="B15" s="12" t="s">
+        <v>212</v>
+      </c>
+      <c r="C15" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="D15" s="18" t="s">
-        <v>206</v>
+      <c r="D15" s="3" t="s">
+        <v>213</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B16" s="17" t="s">
-        <v>207</v>
-      </c>
-      <c r="C16" s="18" t="n">
+      <c r="B16" s="12" t="s">
+        <v>214</v>
+      </c>
+      <c r="C16" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="D16" s="18"/>
+      <c r="D16" s="3"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B17" s="17" t="s">
-        <v>208</v>
-      </c>
-      <c r="C17" s="18" t="n">
+      <c r="B17" s="12" t="s">
+        <v>215</v>
+      </c>
+      <c r="C17" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="D17" s="18" t="s">
-        <v>209</v>
+      <c r="D17" s="3" t="s">
+        <v>216</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B18" s="17" t="s">
-        <v>210</v>
-      </c>
-      <c r="C18" s="18" t="n">
+      <c r="B18" s="12" t="s">
+        <v>217</v>
+      </c>
+      <c r="C18" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="D18" s="18"/>
+      <c r="D18" s="3"/>
     </row>
     <row r="19" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B19" s="17" t="s">
-        <v>211</v>
-      </c>
-      <c r="C19" s="18" t="s">
-        <v>212</v>
-      </c>
-      <c r="D19" s="18" t="s">
-        <v>213</v>
+      <c r="B19" s="12" t="s">
+        <v>218</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>219</v>
+      </c>
+      <c r="D19" s="3" t="s">
+        <v>220</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B20" s="17" t="s">
-        <v>214</v>
-      </c>
-      <c r="C20" s="17" t="s">
-        <v>215</v>
-      </c>
-      <c r="D20" s="18" t="s">
-        <v>216</v>
+      <c r="B20" s="12" t="s">
+        <v>221</v>
+      </c>
+      <c r="C20" s="12" t="s">
+        <v>222</v>
+      </c>
+      <c r="D20" s="3" t="s">
+        <v>223</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="77.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B21" s="17" t="s">
-        <v>217</v>
-      </c>
-      <c r="C21" s="18" t="s">
-        <v>218</v>
+      <c r="B21" s="12" t="s">
+        <v>224</v>
+      </c>
+      <c r="C21" s="3" t="s">
+        <v>225</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="B5:D21"/>
   <mergeCells count="1">
     <mergeCell ref="B3:D3"/>
   </mergeCells>
@@ -3078,5 +3067,6 @@
     <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
     <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
   </headerFooter>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>